<commit_message>
Update Cs-137 reference outputs to 1M events
</commit_message>
<xml_diff>
--- a/results/tables/reference_summary.xlsx
+++ b/results/tables/reference_summary.xlsx
@@ -489,7 +489,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>solid_cs137_10k</t>
+          <t>solid_cs137_1M</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>10000</v>
+        <v>1000000</v>
       </c>
       <c r="F2" t="n">
         <v>662</v>
@@ -517,26 +517,26 @@
         <v>20</v>
       </c>
       <c r="H2" t="n">
-        <v>911</v>
+        <v>92977</v>
       </c>
       <c r="I2" t="n">
-        <v>2047</v>
+        <v>212786</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>results/root/solid_cs137_10k.root</t>
+          <t>results/root/solid_cs137_1M.root</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>results/spectra/solid_cs137_10k.png</t>
+          <t>results/spectra/solid_cs137_1M.png</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>hollow_cs137_10k</t>
+          <t>hollow_cs137_1M</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>10000</v>
+        <v>1000000</v>
       </c>
       <c r="F3" t="n">
         <v>662</v>
@@ -564,26 +564,26 @@
         <v>20</v>
       </c>
       <c r="H3" t="n">
-        <v>4171</v>
+        <v>420750</v>
       </c>
       <c r="I3" t="n">
-        <v>6080</v>
+        <v>616096</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>results/root/hollow_cs137_10k.root</t>
+          <t>results/root/hollow_cs137_1M.root</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>results/spectra/hollow_cs137_10k.png</t>
+          <t>results/spectra/hollow_cs137_1M.png</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>soccerball_cs137_10k</t>
+          <t>soccerball_cs137_1M</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>10000</v>
+        <v>1000000</v>
       </c>
       <c r="F4" t="n">
         <v>662</v>
@@ -611,19 +611,19 @@
         <v>20</v>
       </c>
       <c r="H4" t="n">
-        <v>9449</v>
+        <v>943364</v>
       </c>
       <c r="I4" t="n">
-        <v>9889</v>
+        <v>988303</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>results/root/soccerball_cs137_10k.root</t>
+          <t>results/root/soccerball_cs137_1M.root</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>results/spectra/soccerball_cs137_10k.png</t>
+          <t>results/spectra/soccerball_cs137_1M.png</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>solid_cs137_10k</t>
+          <t>solid_cs137_1M</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -710,29 +710,29 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>10000</v>
+        <v>1000000</v>
       </c>
       <c r="F2" t="n">
-        <v>2047</v>
+        <v>212786</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>results/root/solid_cs137_10k.root</t>
+          <t>results/root/solid_cs137_1M.root</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>results/spectra/solid_cs137_10k.png</t>
+          <t>results/spectra/solid_cs137_1M.png</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>911</v>
+        <v>92977</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>hollow_cs137_10k</t>
+          <t>hollow_cs137_1M</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -751,29 +751,29 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>10000</v>
+        <v>1000000</v>
       </c>
       <c r="F3" t="n">
-        <v>6080</v>
+        <v>616096</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>results/root/hollow_cs137_10k.root</t>
+          <t>results/root/hollow_cs137_1M.root</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>results/spectra/hollow_cs137_10k.png</t>
+          <t>results/spectra/hollow_cs137_1M.png</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>4171</v>
+        <v>420750</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>soccerball_cs137_10k</t>
+          <t>soccerball_cs137_1M</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -792,23 +792,23 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>10000</v>
+        <v>1000000</v>
       </c>
       <c r="F4" t="n">
-        <v>9889</v>
+        <v>988303</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>results/root/soccerball_cs137_10k.root</t>
+          <t>results/root/soccerball_cs137_1M.root</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>results/spectra/soccerball_cs137_10k.png</t>
+          <t>results/spectra/soccerball_cs137_1M.png</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>9449</v>
+        <v>943364</v>
       </c>
     </row>
   </sheetData>

</xml_diff>